<commit_message>
#22 (BOM and Deliverables Updated)
</commit_message>
<xml_diff>
--- a/Design Files/Test Power Module PCB Design v1.0.0/BOM/Test Power Module PCB Design v1.0.0.xlsx
+++ b/Design Files/Test Power Module PCB Design v1.0.0/BOM/Test Power Module PCB Design v1.0.0.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\gerholdvoorde-dronebms\Design Files\Test Power Module PCB Design v1.0.0\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4940623-DC79-4CD0-BB60-82990F25F2EF}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD5AC938-4F5F-4E1A-ABC8-D84D93E02CAC}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="43">
   <si>
     <t>#</t>
   </si>
@@ -34,7 +34,7 @@
     <t>Spacer</t>
   </si>
   <si>
-    <t>Button And Strip Battery Connector</t>
+    <t>Pogo Pin Spring Probe Connector</t>
   </si>
   <si>
     <t>Resistor</t>
@@ -52,7 +52,7 @@
     <t>J2, J3, J4, J5</t>
   </si>
   <si>
-    <t>J6</t>
+    <t>J6, J7, J8, J9, J10</t>
   </si>
   <si>
     <t>R1</t>
@@ -73,7 +73,7 @@
     <t>Spacer Material: Steel Mounting: SMT Series: WA-SMSI Thread D: M2.5</t>
   </si>
   <si>
-    <t>Blade/Shrapnel Connector -40℃~+105℃ Plugin Button And Strip Battery Connector ROHS</t>
+    <t>Brass 12V -40℃~+85℃ 单PINBit 弹簧顶针(POGO PIN) 8.3mm 50mΩ 10000次 4.28mm 2A Gold - Pogo Pin Spring Probe Connector ROHS</t>
   </si>
   <si>
     <t>RES 30K OHM 1% 1/10W 0603</t>
@@ -91,10 +91,10 @@
     <t>HDR1X4 Female</t>
   </si>
   <si>
-    <t>FPG40004-S05S1017M</t>
-  </si>
-  <si>
-    <t>Res-0603</t>
+    <t>YZ162317083P-01</t>
+  </si>
+  <si>
+    <t>RES-0603</t>
   </si>
   <si>
     <t>TL3340AF160QG</t>
@@ -112,7 +112,7 @@
     <t>RT0603BRD0710KL</t>
   </si>
   <si>
-    <t>Manufacturer</t>
+    <t>MANUFACTURER</t>
   </si>
   <si>
     <t>BOOMELE</t>
@@ -121,7 +121,7 @@
     <t>Wurth Electronics</t>
   </si>
   <si>
-    <t>TXGA</t>
+    <t>Xinyangze</t>
   </si>
   <si>
     <t>Yageo</t>
@@ -139,16 +139,13 @@
     <t>Quantity</t>
   </si>
   <si>
+    <t>Remarks</t>
+  </si>
+  <si>
     <t>Value</t>
   </si>
   <si>
-    <t xml:space="preserve"> Remarks</t>
-  </si>
-  <si>
     <t>-</t>
-  </si>
-  <si>
-    <t>RC0603FR-0730KL</t>
   </si>
   <si>
     <t>Custom</t>
@@ -655,8 +652,8 @@
     <col min="7" max="7" width="33.42578125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="21.42578125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="6.140625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="16.7109375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="9" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="8.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -696,13 +693,13 @@
         <v>30</v>
       </c>
       <c r="I2" s="6" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="J2" s="5" t="s">
         <v>38</v>
       </c>
       <c r="K2" s="5" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="3" spans="1:11" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -752,8 +749,8 @@
       <c r="E4" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="F4" s="7" t="s">
-        <v>43</v>
+      <c r="F4" s="9" t="s">
+        <v>42</v>
       </c>
       <c r="G4" s="10" t="s">
         <v>28</v>
@@ -769,7 +766,7 @@
       </c>
       <c r="K4" s="9"/>
     </row>
-    <row r="5" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:11" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1"/>
       <c r="B5" s="11">
         <f>ROW(B5) - ROW($B$2)</f>
@@ -784,8 +781,8 @@
       <c r="E5" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="F5" s="7" t="s">
-        <v>43</v>
+      <c r="F5" s="9" t="s">
+        <v>42</v>
       </c>
       <c r="G5" s="8" t="s">
         <v>23</v>
@@ -797,7 +794,7 @@
         <v>41</v>
       </c>
       <c r="J5" s="7">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="K5" s="7"/>
     </row>
@@ -807,9 +804,7 @@
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="C6" s="12" t="s">
-        <v>5</v>
-      </c>
+      <c r="C6" s="13"/>
       <c r="D6" s="9" t="s">
         <v>11</v>
       </c>
@@ -819,12 +814,8 @@
       <c r="F6" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="G6" s="10" t="s">
-        <v>42</v>
-      </c>
-      <c r="H6" s="7" t="s">
-        <v>34</v>
-      </c>
+      <c r="G6" s="10"/>
+      <c r="H6" s="9"/>
       <c r="I6" s="10" t="s">
         <v>36</v>
       </c>
@@ -880,8 +871,8 @@
       <c r="E8" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="F8" s="7" t="s">
-        <v>43</v>
+      <c r="F8" s="9" t="s">
+        <v>42</v>
       </c>
       <c r="G8" s="10" t="s">
         <v>25</v>

</xml_diff>